<commit_message>
test: finalize phase 0-6 retest and SRS alignment
</commit_message>
<xml_diff>
--- a/07_Testing Plan/PHASE_0_6_AUDIT_TRACKER.xlsx
+++ b/07_Testing Plan/PHASE_0_6_AUDIT_TRACKER.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R3db90fa14a3749e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Guide" sheetId="2" r:id="R14480ebef4144c68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Plan" sheetId="3" r:id="R7e075c8492884a3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carryover P0-4" sheetId="4" r:id="R99f73baa2d3a4da6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 5 Scenarios" sheetId="5" r:id="R8fcb587bff734073"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 6 Scenarios" sheetId="6" r:id="R5e8476ca9bb84f4b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Log" sheetId="7" r:id="R197e2869251342ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Access Baseline" sheetId="8" r:id="Re75317f3513a4573"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4d72942913fb46e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Guide" sheetId="2" r:id="R6ee05831509045b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Plan" sheetId="3" r:id="Rea345a85791b4a0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carryover P0-4" sheetId="4" r:id="R5d1ec4bc22f2446a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 5 Scenarios" sheetId="5" r:id="R10e5619c0d7b4854"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 6 Scenarios" sheetId="6" r:id="R2cd52c230a6f4004"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Log" sheetId="7" r:id="Rd4945925d0404deb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Access Baseline" sheetId="8" r:id="R28fd296d9c2b4f96"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -241,7 +241,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="121">
+  <x:cellXfs count="125">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -519,6 +519,18 @@
     <x:xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -745,7 +757,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>Audit tracker cleaned 2026-08-15: obsolete traced cases removed; P5-RP-001 moved to Future Backlog; P5-PI-011 kept as the sole Not Required case without a DEV action.</x:v>
+        <x:v>Retest finalized 2026-08-17: 32 baseline cases BA-confirmed; GAP-P2-IS-004 added as a separate Dev Owner persistence defect; formulas reflect current scenario statuses.</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -775,14 +787,14 @@
       </x:c>
       <x:c r="B5" s="77" t="n">
         <x:f>COUNTIF('Carryover P0-4'!$L$5:$L$68,A5)+COUNTIF('Phase 5 Scenarios'!$L$5:$L$82,A5)+COUNTIF('Phase 6 Scenarios'!$L$5:$L$57,A5)</x:f>
-        <x:v>120</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="D5" s="77" t="str">
         <x:v>Carryover P0-4</x:v>
       </x:c>
       <x:c r="E5" s="77" t="n">
         <x:f>COUNTA('Carryover P0-4'!$A$5:$A$68)</x:f>
-        <x:v>63</x:v>
+        <x:v>64</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -791,7 +803,7 @@
       </x:c>
       <x:c r="B6" s="77" t="n">
         <x:f>COUNTIF('Carryover P0-4'!$L$5:$L$68,A6)+COUNTIF('Phase 5 Scenarios'!$L$5:$L$82,A6)+COUNTIF('Phase 6 Scenarios'!$L$5:$L$57,A6)</x:f>
-        <x:v>20</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D6" s="77" t="str">
         <x:v>Phase 5 scenarios</x:v>
@@ -807,7 +819,7 @@
       </x:c>
       <x:c r="B7" s="77" t="n">
         <x:f>COUNTIF('Carryover P0-4'!$L$5:$L$68,A7)+COUNTIF('Phase 5 Scenarios'!$L$5:$L$82,A7)+COUNTIF('Phase 6 Scenarios'!$L$5:$L$57,A7)</x:f>
-        <x:v>20</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D7" s="77" t="str">
         <x:v>Phase 6 scenarios</x:v>
@@ -823,14 +835,14 @@
       </x:c>
       <x:c r="B8" s="77" t="n">
         <x:f>COUNTIF('Carryover P0-4'!$L$5:$L$68,A8)+COUNTIF('Phase 5 Scenarios'!$L$5:$L$82,A8)+COUNTIF('Phase 6 Scenarios'!$L$5:$L$57,A8)</x:f>
-        <x:v>17</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D8" s="77" t="str">
         <x:v>Active scenarios</x:v>
       </x:c>
       <x:c r="E8" s="77" t="n">
         <x:f>SUM(E5:E7)-B10-B11</x:f>
-        <x:v>179</x:v>
+        <x:v>180</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -839,7 +851,7 @@
       </x:c>
       <x:c r="B9" s="77" t="n">
         <x:f>COUNTIF('Carryover P0-4'!$L$5:$L$68,A9)+COUNTIF('Phase 5 Scenarios'!$L$5:$L$82,A9)+COUNTIF('Phase 6 Scenarios'!$L$5:$L$57,A9)</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="77"/>
       <x:c r="E9" s="77"/>
@@ -857,7 +869,7 @@
       </x:c>
       <x:c r="E10" s="89" t="n">
         <x:f>IF(E8=0,0,(B5+B6+B7+B8)/E8)</x:f>
-        <x:v>0.9888268156424581</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -889,12 +901,14 @@
         <x:v>Test data</x:v>
       </x:c>
       <x:c r="C14" s="82" t="str">
-        <x:v>AUDIT26 has Milestones, Releases, Features, Work Items, Tasks and report data. A second Team cannot be created because Team lead = Unassigned returns Validation failed.</x:v>
+        <x:v>Controlled TEST/AUDIT26 data covers Releases, Milestones, Portfolio, Work Items, Tasks, multi-Team allocations and Reports.</x:v>
       </x:c>
       <x:c r="D14" s="82" t="str">
-        <x:v>Keeps split-allocation and multi-Team Capacity Planning branches blocked.</x:v>
-      </x:c>
-      <x:c r="E14" s="82"/>
+        <x:v>Remaining blocked cases require finalized daily snapshots or a deliberately invalid acceptedDate fixture.</x:v>
+      </x:c>
+      <x:c r="E14" s="82" t="str">
+        <x:v>Partially ready</x:v>
+      </x:c>
       <x:c r="F14" s="82"/>
       <x:c r="G14" s="82"/>
       <x:c r="H14" s="71"/>
@@ -904,15 +918,17 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B15" s="83" t="str">
-        <x:v>Test accounts</x:v>
+        <x:v>Accounts and roles</x:v>
       </x:c>
       <x:c r="C15" s="83" t="str">
-        <x:v>Workspace Admin plus Project-scoped Admin and Editor sessions are required; include one Project with no assignment.</x:v>
+        <x:v>Workspace Admin, Project Admin, Editor and unassigned/no-access sessions were retested.</x:v>
       </x:c>
       <x:c r="D15" s="83" t="str">
-        <x:v>Blocks current access-level and denied-route proof. Viewer/selectable No Access are Future Backlog.</x:v>
-      </x:c>
-      <x:c r="E15" s="83"/>
+        <x:v>Current RBAC failure is an enforcement defect, not a missing account.</x:v>
+      </x:c>
+      <x:c r="E15" s="83" t="str">
+        <x:v>Ready</x:v>
+      </x:c>
       <x:c r="F15" s="83"/>
       <x:c r="G15" s="83"/>
       <x:c r="H15" s="73"/>
@@ -925,12 +941,14 @@
         <x:v>Notification data</x:v>
       </x:c>
       <x:c r="C16" s="83" t="str">
-        <x:v>Safe recipient and notification rows are required</x:v>
+        <x:v>Controlled assignment and @mention notifications were verified.</x:v>
       </x:c>
       <x:c r="D16" s="83" t="str">
-        <x:v>Carries blocked Phase 4 cases</x:v>
-      </x:c>
-      <x:c r="E16" s="83"/>
+        <x:v>Dev Owner persistence is tracked separately as GAP-P2-IS-004.</x:v>
+      </x:c>
+      <x:c r="E16" s="83" t="str">
+        <x:v>Ready</x:v>
+      </x:c>
       <x:c r="F16" s="83"/>
       <x:c r="G16" s="83"/>
       <x:c r="H16" s="73"/>
@@ -958,6 +976,7 @@
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
     <x:mergeCell ref="A13:H13"/>
+    <x:mergeCell ref="A2:E2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1163,7 +1182,7 @@
         <x:v>BA + Tester</x:v>
       </x:c>
       <x:c r="H5" s="71" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Completed</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -1189,7 +1208,7 @@
         <x:v>BA/User</x:v>
       </x:c>
       <x:c r="H6" s="73" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Completed</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1215,7 +1234,7 @@
         <x:v>BA/User</x:v>
       </x:c>
       <x:c r="H7" s="73" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Completed</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -1241,7 +1260,7 @@
         <x:v>BA/User</x:v>
       </x:c>
       <x:c r="H8" s="73" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Completed</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1267,7 +1286,7 @@
         <x:v>BA/User</x:v>
       </x:c>
       <x:c r="H9" s="73" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Completed</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1371,7 +1390,7 @@
         <x:v>BA</x:v>
       </x:c>
       <x:c r="H13" s="75" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Completed</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1432,7 +1451,7 @@
       <x:c r="O1" s="4"/>
       <x:c r="P1" s="4"/>
       <x:c r="Q1" s="4"/>
-      <x:c r="R1" s="4"/>
+      <x:c r="R1" s="121"/>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="8" t="str">
@@ -1454,7 +1473,10 @@
       <x:c r="O2" s="8"/>
       <x:c r="P2" s="8"/>
       <x:c r="Q2" s="8"/>
-      <x:c r="R2" s="8"/>
+      <x:c r="R2" s="122"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="R3" s="92"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="14" t="str">
@@ -1508,7 +1530,7 @@
       <x:c r="Q4" s="14" t="str">
         <x:v>BA Confirmation</x:v>
       </x:c>
-      <x:c r="R4" s="14" t="str">
+      <x:c r="R4" s="123" t="str">
         <x:v>Test Date</x:v>
       </x:c>
     </x:row>
@@ -2297,25 +2319,25 @@
         <x:v>Deferred (not tested)</x:v>
       </x:c>
       <x:c r="L17" s="51" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M17" s="51" t="str">
-        <x:v>Invite dialog exists but captures email only; no optional Project Access or review step. Delivery was not triggered.</x:v>
+        <x:v>Invite dialog now supports email, role, optional initial Project Access and Review Changes; actual sending is deferred by the approved expected rule.</x:v>
       </x:c>
       <x:c r="N17" s="51" t="str">
         <x:v>https://rally-dev.qnsc.vn/settings</x:v>
       </x:c>
       <x:c r="O17" s="51" t="str">
-        <x:v>Invite dialog exists but captures email only; no optional Project Access or review step. Delivery was not triggered.</x:v>
+        <x:v>Closed after current DevInt retest.</x:v>
       </x:c>
       <x:c r="P17" s="51" t="str">
         <x:v>Codex DevInt retest</x:v>
       </x:c>
       <x:c r="Q17" s="51" t="str">
-        <x:v>Pending BA review</x:v>
-      </x:c>
-      <x:c r="R17" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>Codex retest 2026-08-17</x:v>
+      </x:c>
+      <x:c r="R17" s="56" t="str">
+        <x:v>2026-08-17</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -2924,25 +2946,25 @@
         <x:v>Still Open</x:v>
       </x:c>
       <x:c r="L27" s="51" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M27" s="51" t="str">
-        <x:v>Details, Tasks and Revision History exist, but an extra Connections tab plus Linked Items/Comments remains.</x:v>
+        <x:v>Work Item detail contains the required tabs plus accepted Connections, Linked Items and Comments extensions.</x:v>
       </x:c>
       <x:c r="N27" s="51" t="str">
         <x:v>https://rally-dev.qnsc.vn/item/US-1</x:v>
       </x:c>
       <x:c r="O27" s="51" t="str">
-        <x:v>Details, Tasks and Revision History exist, but an extra Connections tab plus Linked Items/Comments remains.</x:v>
+        <x:v>Closed by BA confirmation; no DEV fix required.</x:v>
       </x:c>
       <x:c r="P27" s="51" t="str">
-        <x:v>Codex DevInt retest</x:v>
+        <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q27" s="51" t="str">
-        <x:v>Pending BA review</x:v>
+        <x:v>BA confirmed 2026-08-17</x:v>
       </x:c>
       <x:c r="R27" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>46251</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -3123,22 +3145,22 @@
         <x:v>Fail</x:v>
       </x:c>
       <x:c r="M30" s="51" t="str">
-        <x:v>BA confirmed live 2026-08-14: Owner selector omits active Work Item Team members.</x:v>
+        <x:v>Owner dropdown on US-1 and TA-1 shows only No Entry although Pegasus has active member Anh.</x:v>
       </x:c>
       <x:c r="N30" s="51" t="str">
         <x:v>https://rally-dev.qnsc.vn/item/US-1</x:v>
       </x:c>
       <x:c r="O30" s="51" t="str">
-        <x:v>Work Item Detail Owner excludes Workspace Admin. BA requires Workspace Admin to remain selectable as Owner without Project/Team membership.</x:v>
+        <x:v>DEV: load Unassigned plus active members of the selected Team; use the same owner candidate source on detail and inline views.</x:v>
       </x:c>
       <x:c r="P30" s="51" t="str">
-        <x:v>Codex DevInt retest</x:v>
+        <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q30" s="51" t="str">
-        <x:v>BA confirmed 2026-08-14</x:v>
+        <x:v>BA confirmed 2026-08-17</x:v>
       </x:c>
       <x:c r="R30" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>46251</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -3635,25 +3657,25 @@
         <x:v>Still Open</x:v>
       </x:c>
       <x:c r="L38" s="51" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M38" s="51" t="str">
-        <x:v>Task history now records Task Created, state and To Do, but Task State events are labelled Schedule State.</x:v>
+        <x:v>Task Revision History now labels every state event as Task State and includes Task Created/To Do history.</x:v>
       </x:c>
       <x:c r="N38" s="51" t="str">
-        <x:v>https://rally-dev.qnsc.vn/item/US-1</x:v>
+        <x:v>https://rally-dev.qnsc.vn/item/TA-1</x:v>
       </x:c>
       <x:c r="O38" s="51" t="str">
-        <x:v>Task history now records Task Created, state and To Do, but Task State events are labelled Schedule State.</x:v>
+        <x:v>Closed after current DevInt retest.</x:v>
       </x:c>
       <x:c r="P38" s="51" t="str">
         <x:v>Codex DevInt retest</x:v>
       </x:c>
       <x:c r="Q38" s="51" t="str">
-        <x:v>Pending BA review</x:v>
-      </x:c>
-      <x:c r="R38" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>Codex retest 2026-08-17</x:v>
+      </x:c>
+      <x:c r="R38" s="56" t="str">
+        <x:v>2026-08-17</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -4266,25 +4288,25 @@
         <x:v>Still Open</x:v>
       </x:c>
       <x:c r="L48" s="51" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M48" s="51" t="str">
-        <x:v>BA confirmed live 2026-08-14: Team Status counts a Task but does not render its Task row/inline State control.</x:v>
+        <x:v>The counted Unassigned task TA-3 renders exactly once after expanding the group and exposes an inline State combobox.</x:v>
       </x:c>
       <x:c r="N48" s="51" t="str">
         <x:v>https://rally-dev.qnsc.vn/team-status</x:v>
       </x:c>
       <x:c r="O48" s="51" t="str">
-        <x:v>Member summary says one Task, but no Task row/inline State dropdown is rendered.</x:v>
+        <x:v>Closed after current DevInt retest.</x:v>
       </x:c>
       <x:c r="P48" s="51" t="str">
         <x:v>Codex DevInt retest</x:v>
       </x:c>
       <x:c r="Q48" s="51" t="str">
-        <x:v>Pending BA review</x:v>
-      </x:c>
-      <x:c r="R48" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>Codex retest 2026-08-17</x:v>
+      </x:c>
+      <x:c r="R48" s="56" t="str">
+        <x:v>2026-08-17</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -4331,25 +4353,25 @@
         <x:v>Still Open</x:v>
       </x:c>
       <x:c r="L49" s="51" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M49" s="51" t="str">
-        <x:v>Totals render, but no empty Task row exists to prove all numeric defaults.</x:v>
+        <x:v>TA-3 shows Estimate 4h, To Do 4h, Actual 0h; dash is used only for missing Owner and empty totals show 0h.</x:v>
       </x:c>
       <x:c r="N49" s="51" t="str">
         <x:v>https://rally-dev.qnsc.vn/team-status</x:v>
       </x:c>
       <x:c r="O49" s="51" t="str">
-        <x:v>Totals render, but no empty Task row exists to prove all numeric defaults.</x:v>
+        <x:v>Closed by BA confirmation; no DEV fix required.</x:v>
       </x:c>
       <x:c r="P49" s="51" t="str">
-        <x:v>Codex DevInt retest</x:v>
+        <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q49" s="51" t="str">
-        <x:v>Pending BA review</x:v>
+        <x:v>BA confirmed 2026-08-17</x:v>
       </x:c>
       <x:c r="R49" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>46251</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -4396,25 +4418,25 @@
         <x:v>Still Open</x:v>
       </x:c>
       <x:c r="L50" s="51" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M50" s="51" t="str">
-        <x:v>BA confirmed live 2026-08-14: counted Task cannot expose the required inline State values because its row is absent.</x:v>
+        <x:v>Inline Task State offers Defined/In-Progress/Completed, persisted In-Progress after reload, and was restored to Defined with reload proof.</x:v>
       </x:c>
       <x:c r="N50" s="51" t="str">
         <x:v>https://rally-dev.qnsc.vn/team-status</x:v>
       </x:c>
       <x:c r="O50" s="51" t="str">
-        <x:v>Counted Task row is absent, so exact editable Task State labels cannot be used.</x:v>
+        <x:v>Closed after current DevInt retest.</x:v>
       </x:c>
       <x:c r="P50" s="51" t="str">
         <x:v>Codex DevInt retest</x:v>
       </x:c>
       <x:c r="Q50" s="51" t="str">
-        <x:v>Pending BA review</x:v>
-      </x:c>
-      <x:c r="R50" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>Codex retest 2026-08-17</x:v>
+      </x:c>
+      <x:c r="R50" s="56" t="str">
+        <x:v>2026-08-17</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -4464,22 +4486,22 @@
         <x:v>Fail</x:v>
       </x:c>
       <x:c r="M51" s="51" t="str">
-        <x:v>BA confirmed live 2026-08-14: Task Roll-up/progress is still shown in Release Detail.</x:v>
+        <x:v>Release RE-2 detail still shows Task Roll-up columns Estimate, To Do, Actual and Accepted.</x:v>
       </x:c>
       <x:c r="N51" s="51" t="str">
-        <x:v>https://rally-dev.qnsc.vn/releases</x:v>
+        <x:v>https://rally-dev.qnsc.vn/releases/019fff28-51be-7024-a876-dd7cc6eb0ec0</x:v>
       </x:c>
       <x:c r="O51" s="51" t="str">
-        <x:v>Release Detail still includes Task Roll-up and Burndown, which Phase 3 defers.</x:v>
+        <x:v>DEV: remove the obsolete Task Roll-up section/columns from Release detail; Release artifact tracking remains the source of truth.</x:v>
       </x:c>
       <x:c r="P51" s="51" t="str">
-        <x:v>Codex DevInt retest</x:v>
+        <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q51" s="51" t="str">
-        <x:v>Pending BA review</x:v>
+        <x:v>BA confirmed 2026-08-17</x:v>
       </x:c>
       <x:c r="R51" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>46251</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -4527,25 +4549,25 @@
         <x:v>Still Open</x:v>
       </x:c>
       <x:c r="L52" s="51" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M52" s="51" t="str">
-        <x:v>Live retest 2026-08-15: Release Add Artifact can add/remove existing US/DE and persists after reload. RE-1 shows its assigned US, but FE-6 still shows RE-2 in Portfolio after reload while RE-2 Artifacts reports 0 items.</x:v>
+        <x:v>Reloaded Release Artifacts shows directly assigned FE-6 exactly once.</x:v>
       </x:c>
       <x:c r="N52" s="51" t="str">
-        <x:v>https://rally-dev.qnsc.vn/releases/019fff28-51be-7024-a876-dd7cc6eb0ec0; https://rally-dev.qnsc.vn/portfolio</x:v>
+        <x:v>https://rally-dev.qnsc.vn/releases/019fff28-51be-7024-a876-dd7cc6eb0ec0</x:v>
       </x:c>
       <x:c r="O52" s="51" t="str">
-        <x:v>Keep the working US/DE assignment behavior and fix Release Artifacts query/display for a directly assigned Feature. Artifact-origin Create/Create with details remains Future Backlog.</x:v>
+        <x:v>Closed after current DevInt retest.</x:v>
       </x:c>
       <x:c r="P52" s="51" t="str">
         <x:v>Codex DevInt retest</x:v>
       </x:c>
       <x:c r="Q52" s="51" t="str">
-        <x:v>BA confirmed Fail 2026-08-15</x:v>
-      </x:c>
-      <x:c r="R52" s="56" t="n">
-        <x:v>46249</x:v>
+        <x:v>Codex retest 2026-08-17</x:v>
+      </x:c>
+      <x:c r="R52" s="56" t="str">
+        <x:v>2026-08-17</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
@@ -4718,25 +4740,25 @@
         <x:v>Blocked (test data)</x:v>
       </x:c>
       <x:c r="L55" s="51" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M55" s="51" t="str">
-        <x:v>Re-tested 2026-08-15: Notification popover still shows 0 of 0. Controlled assignment data could not be generated because the Pegasus Work Item and Task Owner selectors expose only Unassigned / No Entry, and no second sender session is available.</x:v>
+        <x:v>Assignment notifications appear with correct unread state, filters and count.</x:v>
       </x:c>
       <x:c r="N55" s="51" t="str">
-        <x:v>https://rally-dev.qnsc.vn/notifications; https://rally-dev.qnsc.vn/item/US-17</x:v>
+        <x:v>https://rally-dev.qnsc.vn/</x:v>
       </x:c>
       <x:c r="O55" s="51" t="str">
-        <x:v>Retest after active Team members appear in Owner options and a second sender/recipient session is available. Then verify unread count and all four category filters.</x:v>
+        <x:v>Closed by BA confirmation; no DEV fix required.</x:v>
       </x:c>
       <x:c r="P55" s="51" t="str">
-        <x:v>Codex DevInt retest</x:v>
+        <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q55" s="51" t="str">
-        <x:v>Pending BA review</x:v>
+        <x:v>BA confirmed 2026-08-17</x:v>
       </x:c>
       <x:c r="R55" s="56" t="n">
-        <x:v>46249</x:v>
+        <x:v>46251</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -4783,25 +4805,25 @@
         <x:v>Blocked (test data)</x:v>
       </x:c>
       <x:c r="L56" s="51" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M56" s="51" t="str">
-        <x:v>Re-tested 2026-08-15: Notification Center still has no notification row, so single-read and Mark all as read persistence cannot be executed.</x:v>
+        <x:v>Mark one and mark all read persist after reload.</x:v>
       </x:c>
       <x:c r="N56" s="51" t="str">
-        <x:v>https://rally-dev.qnsc.vn/notifications</x:v>
+        <x:v>https://rally-dev.qnsc.vn/</x:v>
       </x:c>
       <x:c r="O56" s="51" t="str">
-        <x:v>Retest immediately after GAP-P4-NOTIF-001 can generate at least two notification rows; verify persistence after reload and sign-in restore.</x:v>
+        <x:v>Closed by BA confirmation; no DEV fix required.</x:v>
       </x:c>
       <x:c r="P56" s="51" t="str">
-        <x:v>Codex DevInt retest</x:v>
+        <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q56" s="51" t="str">
-        <x:v>Pending BA review</x:v>
+        <x:v>BA confirmed 2026-08-17</x:v>
       </x:c>
       <x:c r="R56" s="56" t="n">
-        <x:v>46249</x:v>
+        <x:v>46251</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -4845,25 +4867,25 @@
         <x:v>Blocked (test data)</x:v>
       </x:c>
       <x:c r="L57" s="51" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M57" s="51" t="str">
-        <x:v>No controlled sender/recipient session pair is available.</x:v>
+        <x:v>Owner/Dev Owner assignment and comment @mention notifications route correctly; Dev Owner persistence is tracked separately.</x:v>
       </x:c>
       <x:c r="N57" s="51" t="str">
-        <x:v>https://rally-dev.qnsc.vn/settings</x:v>
+        <x:v>https://rally-dev.qnsc.vn/iteration-status</x:v>
       </x:c>
       <x:c r="O57" s="51" t="str">
-        <x:v>No controlled sender/recipient session pair is available.</x:v>
+        <x:v>Closed by BA confirmation; no DEV fix required.</x:v>
       </x:c>
       <x:c r="P57" s="51" t="str">
-        <x:v>Codex DevInt retest</x:v>
+        <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q57" s="51" t="str">
-        <x:v>Pending BA review</x:v>
+        <x:v>BA confirmed 2026-08-17</x:v>
       </x:c>
       <x:c r="R57" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>46251</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -4904,25 +4926,25 @@
         <x:v>Superseded by approved Project access baseline 2026-08-14; previous permission result cannot be reused.</x:v>
       </x:c>
       <x:c r="L58" s="51" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M58" s="51" t="str">
-        <x:v>WA General is read-only, but WA Project Access still exposes Add project access.</x:v>
+        <x:v>Workspace Admin General and Project Access are both read-only; Add project access is absent and explanatory text confirms global access.</x:v>
       </x:c>
       <x:c r="N58" s="51" t="str">
         <x:v>https://rally-dev.qnsc.vn/settings</x:v>
       </x:c>
       <x:c r="O58" s="51" t="str">
-        <x:v>WA General is read-only, but WA Project Access still exposes Add project access.</x:v>
+        <x:v>Closed after current DevInt retest.</x:v>
       </x:c>
       <x:c r="P58" s="51" t="str">
         <x:v>Codex DevInt retest</x:v>
       </x:c>
       <x:c r="Q58" s="51" t="str">
-        <x:v>Pending BA review</x:v>
-      </x:c>
-      <x:c r="R58" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>Codex retest 2026-08-17</x:v>
+      </x:c>
+      <x:c r="R58" s="56" t="str">
+        <x:v>2026-08-17</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
@@ -4963,25 +4985,25 @@
         <x:v>Superseded by approved Project access baseline 2026-08-14; previous permission result cannot be reused.</x:v>
       </x:c>
       <x:c r="L59" s="51" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Fail</x:v>
       </x:c>
       <x:c r="M59" s="51" t="str">
-        <x:v>Editor and unassigned records exist, but no Admin session and no alternate Editor/unassigned login are available.</x:v>
+        <x:v>Admin path passes, but Editor with no Team can see All Teams/project items; unassigned session exposes aggregate/stale context and detail can render blank.</x:v>
       </x:c>
       <x:c r="N59" s="51" t="str">
-        <x:v>https://rally-dev.qnsc.vn/settings</x:v>
+        <x:v>https://rally-dev.qnsc.vn/backlog</x:v>
       </x:c>
       <x:c r="O59" s="51" t="str">
-        <x:v>Editor and unassigned records exist, but no Admin session and no alternate Editor/unassigned login are available.</x:v>
+        <x:v>DEV: enforce Project/Team scope on API and UI queries; unassigned/no-access users must not receive project data, stale context or blank detail shells.</x:v>
       </x:c>
       <x:c r="P59" s="51" t="str">
-        <x:v>Codex DevInt retest</x:v>
+        <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q59" s="51" t="str">
-        <x:v>Pending BA review</x:v>
+        <x:v>BA confirmed 2026-08-17</x:v>
       </x:c>
       <x:c r="R59" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>46251</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
@@ -5090,25 +5112,25 @@
         <x:v>Still Open</x:v>
       </x:c>
       <x:c r="L61" s="51" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M61" s="51" t="str">
-        <x:v>User list scope is accepted. User Detail, Project Access and role-specific actions remain pending the Admin/Editor/unassigned account set.</x:v>
+        <x:v>Settings access and Editor Team Status read-only behavior match the confirmed role rules; restricted routes remain denied.</x:v>
       </x:c>
       <x:c r="N61" s="51" t="str">
-        <x:v>../Codex_audit_06_tracker.md; https://rally-dev.qnsc.vn/settings</x:v>
+        <x:v>https://rally-dev.qnsc.vn/settings</x:v>
       </x:c>
       <x:c r="O61" s="51" t="str">
-        <x:v>Retest with the approved RBAC account set before closure.</x:v>
+        <x:v>Closed by BA confirmation; no DEV fix required.</x:v>
       </x:c>
       <x:c r="P61" s="51" t="str">
         <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q61" s="51" t="str">
-        <x:v>BA confirmed Partial 2026-08-14</x:v>
+        <x:v>BA confirmed 2026-08-17</x:v>
       </x:c>
       <x:c r="R61" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>46251</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
@@ -5155,25 +5177,25 @@
         <x:v>Still Open</x:v>
       </x:c>
       <x:c r="L62" s="51" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M62" s="51" t="str">
-        <x:v>Team deactivation and Project-access removal have clear confirmation; company-user removal is unavailable.</x:v>
+        <x:v>Destructive confirmation modals work with typed confirmation; minor Deactive copy does not block the flow.</x:v>
       </x:c>
       <x:c r="N62" s="51" t="str">
         <x:v>https://rally-dev.qnsc.vn/settings</x:v>
       </x:c>
       <x:c r="O62" s="51" t="str">
-        <x:v>Team deactivation and Project-access removal have clear confirmation; company-user removal is unavailable.</x:v>
+        <x:v>Closed by BA confirmation; no DEV fix required.</x:v>
       </x:c>
       <x:c r="P62" s="51" t="str">
-        <x:v>Codex DevInt retest</x:v>
+        <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q62" s="51" t="str">
-        <x:v>Pending BA review</x:v>
+        <x:v>BA confirmed 2026-08-17</x:v>
       </x:c>
       <x:c r="R62" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>46251</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
@@ -5281,25 +5303,25 @@
         <x:v>New defect found 2026-08-06</x:v>
       </x:c>
       <x:c r="L64" s="53" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M64" s="53" t="str">
-        <x:v>BA confirmed live 2026-08-14: Team Status member scope is inconsistent with selected Team membership.</x:v>
+        <x:v>Pegasus scope shows active member Anh plus Unassigned only; prior outside-Team Hieu group is absent.</x:v>
       </x:c>
       <x:c r="N64" s="53" t="str">
         <x:v>https://rally-dev.qnsc.vn/team-status</x:v>
       </x:c>
       <x:c r="O64" s="53" t="str">
-        <x:v>Settings lists only Anh in Pegasus while Team Status still groups non-member Hieu with one Task.</x:v>
+        <x:v>Closed after current DevInt retest.</x:v>
       </x:c>
       <x:c r="P64" s="53" t="str">
         <x:v>Codex DevInt retest</x:v>
       </x:c>
       <x:c r="Q64" s="53" t="str">
-        <x:v>Pending BA review</x:v>
-      </x:c>
-      <x:c r="R64" s="57" t="n">
-        <x:v>46248</x:v>
+        <x:v>Codex retest 2026-08-17</x:v>
+      </x:c>
+      <x:c r="R64" s="57" t="str">
+        <x:v>2026-08-17</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
@@ -5339,25 +5361,25 @@
         <x:v>New live audit gap 2026-08-14</x:v>
       </x:c>
       <x:c r="L65" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M65" t="str">
-        <x:v>DevInt still shows Manage Projects at the bottom of the Project/Team dropdown.</x:v>
+        <x:v>Home context selector on 2026-08-17 lists workspace/projects/teams only; Manage Projects is absent.</x:v>
       </x:c>
       <x:c r="N65" t="str">
-        <x:v>../Codex_audit_06_tracker.md; https://rally-dev.qnsc.vn/</x:v>
+        <x:v>https://rally-dev.qnsc.vn/</x:v>
       </x:c>
       <x:c r="O65" t="str">
-        <x:v>Remove Manage Projects from the selector. Keep Project administration under Settings gear only.</x:v>
+        <x:v>Closed after current DevInt retest.</x:v>
       </x:c>
       <x:c r="P65" t="str">
         <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q65" t="str">
-        <x:v>BA confirmed Fail 2026-08-14</x:v>
-      </x:c>
-      <x:c r="R65" s="92" t="n">
-        <x:v>46248</x:v>
+        <x:v>Codex retest 2026-08-17</x:v>
+      </x:c>
+      <x:c r="R65" s="92" t="str">
+        <x:v>2026-08-17</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
@@ -5418,7 +5440,7 @@
       <x:c r="Q66" t="str">
         <x:v>Confirmed Future Backlog 2026-08-15</x:v>
       </x:c>
-      <x:c r="R66" t="n">
+      <x:c r="R66" s="92" t="n">
         <x:v>46249</x:v>
       </x:c>
     </x:row>
@@ -5463,46 +5485,86 @@
         <x:v>Not Run after scope amendment 2026-08-15</x:v>
       </x:c>
       <x:c r="L67" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="M67" t="str">
+        <x:v>Milestone MS-1 shows FE-6, descendant US-8/US-9 and US-18 once after assignment; no duplicate artifact row.</x:v>
+      </x:c>
+      <x:c r="N67" t="str">
+        <x:v>https://rally-dev.qnsc.vn/milestones/019fff28-b5b6-714d-a7e4-f05cbd5430c5</x:v>
+      </x:c>
+      <x:c r="O67" t="str">
+        <x:v>Closed by BA confirmation; no DEV fix required.</x:v>
+      </x:c>
+      <x:c r="P67" t="str">
+        <x:v>BA + Codex</x:v>
+      </x:c>
+      <x:c r="Q67" t="str">
+        <x:v>BA confirmed 2026-08-17</x:v>
+      </x:c>
+      <x:c r="R67" s="92" t="n">
+        <x:v>46251</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" t="str">
+        <x:v>GAP-P2-IS-004</x:v>
+      </x:c>
+      <x:c r="B68" t="str">
+        <x:v>Phase 2</x:v>
+      </x:c>
+      <x:c r="C68" t="str">
+        <x:v>Iteration Status - inline Dev Owner</x:v>
+      </x:c>
+      <x:c r="D68" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="E68" t="str">
+        <x:v>Verify inline Dev Owner persists after refresh and is consistent across views.</x:v>
+      </x:c>
+      <x:c r="F68" t="str">
+        <x:v>Authorized user; Work Item assigned to an Iteration; active assignable Team member exists.</x:v>
+      </x:c>
+      <x:c r="G68" t="str">
+        <x:v>Project TEST; one US/DE in selected Iteration; vuhieu24042000 or another active Team member.</x:v>
+      </x:c>
+      <x:c r="H68" t="str">
+        <x:v>1. Open Iteration Status.
+2. Inline-select Dev Owner.
+3. Verify save/notification.
+4. Reload the page.
+5. Reopen the same Work Item/detail.</x:v>
+      </x:c>
+      <x:c r="I68" t="str">
+        <x:v>Selected Dev Owner persists after reload and is consistent in inline/detail views; one notification is emitted for the successful assignment.</x:v>
+      </x:c>
+      <x:c r="J68" t="str">
+        <x:v>Phase 2 Iteration Status SRS: P2-IS-FR-032B, P2-IS-FR-032C</x:v>
+      </x:c>
+      <x:c r="K68" t="str">
+        <x:v>New defect found during 2026-08-17 retest.</x:v>
+      </x:c>
+      <x:c r="L68" t="str">
         <x:v>Fail</x:v>
       </x:c>
-      <x:c r="M67" t="str">
-        <x:v>Live retest 2026-08-15: Milestone Add Artifact can add/remove existing US/DE and persists after reload. FE-6 retains MS-1 after Save/reload, but MS-1 Artifacts still shows only US-8 and US-9; FE-6 is absent. Direct Feature display failed, so inherited Feature/Epic scope cannot be accepted.</x:v>
-      </x:c>
-      <x:c r="N67" t="str">
-        <x:v>https://rally-dev.qnsc.vn/milestones/019fff28-b5b6-714d-a7e4-f05cbd5430c5; https://rally-dev.qnsc.vn/portfolio</x:v>
-      </x:c>
-      <x:c r="O67" t="str">
-        <x:v>Fix Milestone Artifacts query/display for directly assigned Feature/Epic and de-duplicated inherited descendants. Keep existing US/DE behavior. Artifact-origin Create/Create with details remains Future Backlog.</x:v>
-      </x:c>
-      <x:c r="P67" t="str">
-        <x:v>Codex DevInt retest</x:v>
-      </x:c>
-      <x:c r="Q67" t="str">
-        <x:v>BA confirmed Fail 2026-08-15</x:v>
-      </x:c>
-      <x:c r="R67" t="n">
-        <x:v>46249</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="68">
-      <x:c r="A68"/>
-      <x:c r="B68"/>
-      <x:c r="C68"/>
-      <x:c r="D68"/>
-      <x:c r="E68"/>
-      <x:c r="F68"/>
-      <x:c r="G68"/>
-      <x:c r="H68"/>
-      <x:c r="I68"/>
-      <x:c r="J68"/>
-      <x:c r="K68"/>
-      <x:c r="L68"/>
-      <x:c r="M68"/>
-      <x:c r="N68"/>
-      <x:c r="O68"/>
-      <x:c r="P68"/>
-      <x:c r="Q68"/>
-      <x:c r="R68"/>
+      <x:c r="M68" t="str">
+        <x:v>Inline selector accepts the user and notification fires, but after reload Dev Owner returns to No Entry.</x:v>
+      </x:c>
+      <x:c r="N68" t="str">
+        <x:v>https://rally-dev.qnsc.vn/iteration-status</x:v>
+      </x:c>
+      <x:c r="O68" t="str">
+        <x:v>DEV: persist Dev Owner server-side/shared source and reload it consistently; do not emit duplicate notifications.</x:v>
+      </x:c>
+      <x:c r="P68" t="str">
+        <x:v>BA + Codex</x:v>
+      </x:c>
+      <x:c r="Q68" t="str">
+        <x:v>BA confirmed 2026-08-17</x:v>
+      </x:c>
+      <x:c r="R68" s="92" t="n">
+        <x:v>46251</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5813,22 +5875,22 @@
         <x:v>Fail</x:v>
       </x:c>
       <x:c r="M7" s="51" t="str">
-        <x:v>Project must be inherited from the active context and read-only. DevInt exposes an interactive Project selector; selecting AUDIT26 returns an unexpected error.</x:v>
+        <x:v>Feature child creation from FE-6 exposes Project dropdown values TEST, AUDIT26 and P6RT014 instead of inheriting the current Project.</x:v>
       </x:c>
       <x:c r="N7" s="51" t="str">
-        <x:v>../Codex_audit_06_tracker.md; https://rally-dev.qnsc.vn/portfolio</x:v>
+        <x:v>https://rally-dev.qnsc.vn/portfolio/019fff2d-06d7-7956-9ee1-85d45b36ec0c</x:v>
       </x:c>
       <x:c r="O7" s="51" t="str">
-        <x:v>Remove the editable Project selector and always inherit the current Project context.</x:v>
+        <x:v>DEV: Project is inherited from the current context and read-only for all create/detail journeys, including Add Child/Create with detail.</x:v>
       </x:c>
       <x:c r="P7" s="51" t="str">
         <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q7" s="51" t="str">
-        <x:v>BA confirmed Fail 2026-08-14</x:v>
+        <x:v>BA confirmed 2026-08-17</x:v>
       </x:c>
       <x:c r="R7" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>46251</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -5869,25 +5931,25 @@
         <x:v>Superseded by approved Project access baseline 2026-08-14; previous permission result cannot be reused.</x:v>
       </x:c>
       <x:c r="L8" s="51" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M8" s="51" t="str">
-        <x:v>No assigned-Project Admin login is available.</x:v>
+        <x:v>Project Admin can create, edit and archive Features in the assigned Project.</x:v>
       </x:c>
       <x:c r="N8" s="51" t="str">
         <x:v>https://rally-dev.qnsc.vn/portfolio</x:v>
       </x:c>
       <x:c r="O8" s="51" t="str">
-        <x:v>No assigned-Project Admin login is available.</x:v>
+        <x:v>Closed by BA confirmation; no DEV fix required.</x:v>
       </x:c>
       <x:c r="P8" s="51" t="str">
-        <x:v>Codex DevInt retest</x:v>
+        <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q8" s="51" t="str">
-        <x:v>Pending BA review</x:v>
+        <x:v>BA confirmed 2026-08-17</x:v>
       </x:c>
       <x:c r="R8" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>46251</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -5928,25 +5990,25 @@
         <x:v>Superseded by approved Project access baseline 2026-08-14; previous permission result cannot be reused.</x:v>
       </x:c>
       <x:c r="L9" s="51" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M9" s="51" t="str">
-        <x:v>No second unassigned Project and no unassigned-user login are available.</x:v>
+        <x:v>Portfolio data is isolated to the Project assigned to the current user.</x:v>
       </x:c>
       <x:c r="N9" s="51" t="str">
         <x:v>https://rally-dev.qnsc.vn/portfolio</x:v>
       </x:c>
       <x:c r="O9" s="51" t="str">
-        <x:v>No second unassigned Project and no unassigned-user login are available.</x:v>
+        <x:v>Closed by BA confirmation; no DEV fix required.</x:v>
       </x:c>
       <x:c r="P9" s="51" t="str">
-        <x:v>Codex DevInt retest</x:v>
+        <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q9" s="51" t="str">
-        <x:v>Pending BA review</x:v>
+        <x:v>BA confirmed 2026-08-17</x:v>
       </x:c>
       <x:c r="R9" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>46251</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -5987,25 +6049,25 @@
         <x:v>Superseded by approved Project access baseline 2026-08-14; previous permission result cannot be reused.</x:v>
       </x:c>
       <x:c r="L10" s="51" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M10" s="51" t="str">
-        <x:v>No Editor login is available to verify hidden navigation and direct-route denial.</x:v>
+        <x:v>Editor Portfolio menu is hidden and direct Portfolio routes are denied.</x:v>
       </x:c>
       <x:c r="N10" s="51" t="str">
         <x:v>https://rally-dev.qnsc.vn/portfolio</x:v>
       </x:c>
       <x:c r="O10" s="51" t="str">
-        <x:v>No Editor login is available to verify hidden navigation and direct-route denial.</x:v>
+        <x:v>Closed by BA confirmation; no DEV fix required.</x:v>
       </x:c>
       <x:c r="P10" s="51" t="str">
-        <x:v>Codex DevInt retest</x:v>
+        <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q10" s="51" t="str">
-        <x:v>Pending BA review</x:v>
+        <x:v>BA confirmed 2026-08-17</x:v>
       </x:c>
       <x:c r="R10" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>46251</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -6491,25 +6553,25 @@
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="L18" s="51" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M18" s="51" t="str">
-        <x:v>Children uses the Backlog-like grid and expands Work Items, but available child US-5 has no Task rows to verify read-only behavior.</x:v>
+        <x:v>Children uses Backlog-style grid; US-9 expands and TA-2 Task row is rendered read-only while Work Item row remains editable.</x:v>
       </x:c>
       <x:c r="N18" s="51" t="str">
-        <x:v>https://rally-dev.qnsc.vn/portfolio</x:v>
+        <x:v>https://rally-dev.qnsc.vn/portfolio/019fff2d-06d7-7956-9ee1-85d45b36ec0c</x:v>
       </x:c>
       <x:c r="O18" s="51" t="str">
-        <x:v>Children uses the Backlog-like grid and expands Work Items, but available child US-5 has no Task rows to verify read-only behavior.</x:v>
+        <x:v>Closed after current DevInt retest.</x:v>
       </x:c>
       <x:c r="P18" s="51" t="str">
         <x:v>Codex DevInt retest</x:v>
       </x:c>
       <x:c r="Q18" s="51" t="str">
-        <x:v>Pending BA review</x:v>
-      </x:c>
-      <x:c r="R18" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>Codex retest 2026-08-17</x:v>
+      </x:c>
+      <x:c r="R18" s="56" t="str">
+        <x:v>2026-08-17</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -6611,25 +6673,25 @@
         <x:v>Superseded by approved Project access baseline 2026-08-14; previous permission result cannot be reused.</x:v>
       </x:c>
       <x:c r="L20" s="51" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M20" s="51" t="str">
-        <x:v>DevInt Portfolio route loads and Workspace Admin access works; alternate access boundaries and deployment build evidence are unavailable.</x:v>
+        <x:v>Portfolio list/detail loads for Workspace Admin and Project Admin; Editor/unassigned access is denied with project isolation.</x:v>
       </x:c>
       <x:c r="N20" s="51" t="str">
         <x:v>https://rally-dev.qnsc.vn/portfolio</x:v>
       </x:c>
       <x:c r="O20" s="51" t="str">
-        <x:v>DevInt Portfolio route loads and Workspace Admin access works; alternate access boundaries and deployment build evidence are unavailable.</x:v>
+        <x:v>Closed by BA confirmation; no DEV fix required.</x:v>
       </x:c>
       <x:c r="P20" s="51" t="str">
-        <x:v>Codex DevInt retest</x:v>
+        <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q20" s="51" t="str">
-        <x:v>Pending BA review</x:v>
+        <x:v>BA confirmed 2026-08-17</x:v>
       </x:c>
       <x:c r="R20" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>46251</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -6675,25 +6737,25 @@
         <x:v>Pass (runtime smoke 2026-07-26: FE-315 created US-4822 via shared Add Item flow and detail showed FE-315)</x:v>
       </x:c>
       <x:c r="L21" s="51" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M21" s="51" t="str">
-        <x:v>BA confirmed live 2026-08-14: Create works but Create with details cannot complete/open the created detail flow.</x:v>
+        <x:v>Create with details created exactly one US-18, opened that same Detail, prefilled Feature FE-6, and FE-6 Children count reloaded from 1 to 2.</x:v>
       </x:c>
       <x:c r="N21" s="51" t="str">
-        <x:v>https://rally-dev.qnsc.vn/portfolio</x:v>
+        <x:v>https://rally-dev.qnsc.vn/item/US-18</x:v>
       </x:c>
       <x:c r="O21" s="51" t="str">
-        <x:v>`Add New` from FE-2 Children opens the shared New Work Item dialog without a Feature field or FE-2 prefill.</x:v>
+        <x:v>Closed after current DevInt retest.</x:v>
       </x:c>
       <x:c r="P21" s="51" t="str">
         <x:v>Codex DevInt retest</x:v>
       </x:c>
       <x:c r="Q21" s="51" t="str">
-        <x:v>Pending BA review</x:v>
-      </x:c>
-      <x:c r="R21" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>Codex retest 2026-08-17</x:v>
+      </x:c>
+      <x:c r="R21" s="56" t="str">
+        <x:v>2026-08-17</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -6738,25 +6800,25 @@
         <x:v>Partial Pass (runtime smoke 2026-07-26: same-Project active Feature options and selected value verified; Project-change invalid-clear remains BA/UAT Not Run)</x:v>
       </x:c>
       <x:c r="L22" s="51" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M22" s="51" t="str">
-        <x:v>Feature selection persists in Work Item Detail, but the inverse Feature/Epic Children relation is inconsistent for US-5 and US-12.</x:v>
+        <x:v>US-18 Detail shows Feature FE-6 and FE-6 Children reload shows the same new relation.</x:v>
       </x:c>
       <x:c r="N22" s="51" t="str">
-        <x:v>../Codex_audit_06_tracker.md; https://rally-dev.qnsc.vn/item/US-12; https://rally-dev.qnsc.vn/portfolio</x:v>
+        <x:v>https://rally-dev.qnsc.vn/item/US-18</x:v>
       </x:c>
       <x:c r="O22" s="51" t="str">
-        <x:v>Synchronize Work Item Feature assignment with the Feature/Epic Children projection.</x:v>
+        <x:v>Closed after current DevInt retest.</x:v>
       </x:c>
       <x:c r="P22" s="51" t="str">
         <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q22" s="51" t="str">
-        <x:v>BA confirmed Fail 2026-08-14</x:v>
-      </x:c>
-      <x:c r="R22" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>Codex retest 2026-08-17</x:v>
+      </x:c>
+      <x:c r="R22" s="56" t="str">
+        <x:v>2026-08-17</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -6988,23 +7050,25 @@
         <x:v>Historical smoke 2026-07-26 observed auto-zero To Do; superseded by BA rule 2026-08-14.</x:v>
       </x:c>
       <x:c r="L26" s="51" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M26" s="51" t="str">
-        <x:v>Business rule updated 2026-08-14; prior Pass based on auto-zero To Do is superseded and this case requires retest.</x:v>
+        <x:v>Controlled edit persisted Estimate=4, To Do=1 and Actual=2 independently after reload; then restored To Do=0 and Actual=0.</x:v>
       </x:c>
       <x:c r="N26" s="51" t="str">
-        <x:v>DevInt browser retest 2026-08-06; controlled P56-AUDIT data. Detail: 07_Testing Plan/Codex_audit_06_tracker.md &gt; Phase 5 DevInt Execution Results.</x:v>
-      </x:c>
-      <x:c r="O26" s="51"/>
+        <x:v>https://rally-dev.qnsc.vn/item/TA-1</x:v>
+      </x:c>
+      <x:c r="O26" s="51" t="str">
+        <x:v>Closed after current DevInt retest.</x:v>
+      </x:c>
       <x:c r="P26" s="51" t="str">
         <x:v>Codex — Workspace Admin</x:v>
       </x:c>
       <x:c r="Q26" s="51" t="str">
-        <x:v>Pending BA confirmation</x:v>
-      </x:c>
-      <x:c r="R26" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>Codex retest 2026-08-17</x:v>
+      </x:c>
+      <x:c r="R26" s="56" t="str">
+        <x:v>2026-08-17</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -7356,25 +7420,25 @@
         <x:v>Pass / BA accepted 2026-07-28.</x:v>
       </x:c>
       <x:c r="L32" s="51" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M32" s="51" t="str">
-        <x:v>Epic/Feature Children and Work Item Detail disagree on the leaf set, so Epic progress numerators and denominators cannot be trusted.</x:v>
+        <x:v>TEST Epic EP-1 rolls up the same single leaf Work Item as FE-2: 0/3 accepted points and 0/1 accepted items.</x:v>
       </x:c>
       <x:c r="N32" s="51" t="str">
-        <x:v>../Codex_audit_06_tracker.md; https://rally-dev.qnsc.vn/portfolio</x:v>
+        <x:v>https://rally-dev.qnsc.vn/portfolio</x:v>
       </x:c>
       <x:c r="O32" s="51" t="str">
-        <x:v>Fix the hierarchy leaf set before retesting Epic progress formulas.</x:v>
+        <x:v>Closed after current DevInt retest.</x:v>
       </x:c>
       <x:c r="P32" s="51" t="str">
         <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q32" s="51" t="str">
-        <x:v>BA confirmed Fail 2026-08-14</x:v>
-      </x:c>
-      <x:c r="R32" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>Codex retest 2026-08-17</x:v>
+      </x:c>
+      <x:c r="R32" s="56" t="str">
+        <x:v>2026-08-17</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -8104,25 +8168,25 @@
         <x:v>Pending re-smoke</x:v>
       </x:c>
       <x:c r="L44" s="51" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M44" s="51" t="str">
-        <x:v>Add/Remove Teams exposes only Pegasus and another eligible Team cannot be added. This blocks the split-allocation chain.</x:v>
+        <x:v>Created eligible Team Retest Capacity, added it to the plan, then removed it; Team row disappeared and FE-4 returned to Not assigned after reload.</x:v>
       </x:c>
       <x:c r="N44" s="51" t="str">
-        <x:v>../Codex_audit_06_tracker.md; https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
+        <x:v>https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
       </x:c>
       <x:c r="O44" s="51" t="str">
-        <x:v>Root defect for P5-CP-008 and the cross-Team branch of P5-CP-025. Fix Team eligibility/addition and retest.</x:v>
+        <x:v>Closed after current DevInt retest.</x:v>
       </x:c>
       <x:c r="P44" s="51" t="str">
         <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q44" s="51" t="str">
-        <x:v>BA confirmed Fail 2026-08-14</x:v>
-      </x:c>
-      <x:c r="R44" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>Codex retest 2026-08-17</x:v>
+      </x:c>
+      <x:c r="R44" s="56" t="str">
+        <x:v>2026-08-17</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -8229,25 +8293,25 @@
         <x:v>Pending re-smoke</x:v>
       </x:c>
       <x:c r="L46" s="51" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M46" s="51" t="str">
-        <x:v>Split allocation requires two Teams. The second Team cannot be created because Team lead = Unassigned is rejected by validation.</x:v>
+        <x:v>FE-2 split successfully across Pegasus (8) and Retest Capacity (2); plan showed 2 teams and both Team rows.</x:v>
       </x:c>
       <x:c r="N46" s="51" t="str">
-        <x:v>DEVINT_RETEST_EXECUTION_PLAN_2026-08-14.md §8; https://rally-dev.qnsc.vn/settings</x:v>
+        <x:v>https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
       </x:c>
       <x:c r="O46" s="51" t="str">
-        <x:v>Blocked by the Team creation defect; retest after optional Team lead is accepted.</x:v>
+        <x:v>Closed after current DevInt retest.</x:v>
       </x:c>
       <x:c r="P46" s="51" t="str">
         <x:v>Codex DevInt retest</x:v>
       </x:c>
       <x:c r="Q46" s="51" t="str">
-        <x:v>Pending BA review</x:v>
-      </x:c>
-      <x:c r="R46" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>Codex retest 2026-08-17</x:v>
+      </x:c>
+      <x:c r="R46" s="56" t="str">
+        <x:v>2026-08-17</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -8353,25 +8417,25 @@
         <x:v>Pass 2026-07-27: browser smoke verified tooltip content by focus/click interaction. Re-smoked 2026-07-28 under P5-CP-030 for fixed overlay and warnings</x:v>
       </x:c>
       <x:c r="L48" s="51" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="M48" s="51" t="str">
-        <x:v>The in-app test session cannot trigger/hold the required pointer-hover tooltips; visible Breakdown is recorded separately under P5-CP-033.</x:v>
+        <x:v>Team/Feature progress and tooltip are visible and not clipped, but displayed values are incorrect because feature rollup remains 0.</x:v>
       </x:c>
       <x:c r="N48" s="51" t="str">
         <x:v>https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
       </x:c>
       <x:c r="O48" s="51" t="str">
-        <x:v>The in-app test session cannot trigger/hold the required pointer-hover tooltips; visible Breakdown is recorded separately under P5-CP-033.</x:v>
+        <x:v>DEV: keep the current UI; close after P5-CP-029 rollup data is corrected and the tooltip reflects the recalculated values.</x:v>
       </x:c>
       <x:c r="P48" s="51" t="str">
-        <x:v>Codex DevInt retest</x:v>
+        <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q48" s="51" t="str">
-        <x:v>Pending BA review</x:v>
+        <x:v>BA confirmed 2026-08-17</x:v>
       </x:c>
       <x:c r="R48" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>46251</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -8479,25 +8543,25 @@
         <x:v>Pending browser smoke after record-detail v2</x:v>
       </x:c>
       <x:c r="L50" s="51" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M50" s="51" t="str">
-        <x:v>Cutline, Estimated warning and non-Rank hiding pass. Split-Team branch still requires a second Team.</x:v>
+        <x:v>Previously passing cutline/warning/sort branches remain intact; newly unblocked split-Team branch rendered FE-2 under both Teams.</x:v>
       </x:c>
       <x:c r="N50" s="51" t="str">
-        <x:v>../Codex_audit_06_tracker.md; https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
+        <x:v>https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
       </x:c>
       <x:c r="O50" s="51" t="str">
-        <x:v>Retest only the split-Team branch after P5-CP-006 is fixed.</x:v>
+        <x:v>Closed after current DevInt retest.</x:v>
       </x:c>
       <x:c r="P50" s="51" t="str">
         <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q50" s="51" t="str">
-        <x:v>BA confirmed Partial 2026-08-14</x:v>
-      </x:c>
-      <x:c r="R50" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>Codex retest 2026-08-17</x:v>
+      </x:c>
+      <x:c r="R50" s="56" t="str">
+        <x:v>2026-08-17</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -8786,25 +8850,25 @@
         <x:v>Superseded by approved Project access baseline 2026-08-14; previous permission result cannot be reused.</x:v>
       </x:c>
       <x:c r="L55" s="51" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M55" s="51" t="str">
-        <x:v>Only Workspace Admin session is available; Admin, Editor and unassigned boundaries cannot be verified.</x:v>
+        <x:v>Workspace Admin and Project Admin can access Capacity Planning; Editor and unassigned users are denied.</x:v>
       </x:c>
       <x:c r="N55" s="51" t="str">
         <x:v>https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
       </x:c>
       <x:c r="O55" s="51" t="str">
-        <x:v>Only Workspace Admin session is available; Admin, Editor and unassigned boundaries cannot be verified.</x:v>
+        <x:v>Closed by BA confirmation; no DEV fix required.</x:v>
       </x:c>
       <x:c r="P55" s="51" t="str">
-        <x:v>Codex DevInt retest</x:v>
+        <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q55" s="51" t="str">
-        <x:v>Pending BA review</x:v>
+        <x:v>BA confirmed 2026-08-17</x:v>
       </x:c>
       <x:c r="R55" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>46251</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -8849,25 +8913,25 @@
         <x:v>Pass (build + runtime smoke 2026-07-26; Vite chunk-size warning only)</x:v>
       </x:c>
       <x:c r="L56" s="51" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M56" s="51" t="str">
-        <x:v>Capacity Planning route and CP-1 load without a visible fatal UI error; deployment build/console evidence is outside this UI-only retest.</x:v>
+        <x:v>Capacity Planning route and plan views load without crash; rollup correctness is tracked separately.</x:v>
       </x:c>
       <x:c r="N56" s="51" t="str">
         <x:v>https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
       </x:c>
       <x:c r="O56" s="51" t="str">
-        <x:v>Capacity Planning route and CP-1 load without a visible fatal UI error; deployment build/console evidence is outside this UI-only retest.</x:v>
+        <x:v>Closed by BA confirmation; no DEV fix required.</x:v>
       </x:c>
       <x:c r="P56" s="51" t="str">
-        <x:v>Codex DevInt retest</x:v>
+        <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q56" s="51" t="str">
-        <x:v>Pending BA review</x:v>
+        <x:v>BA confirmed 2026-08-17</x:v>
       </x:c>
       <x:c r="R56" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>46251</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -8908,25 +8972,25 @@
         <x:v>Superseded by approved Project access baseline 2026-08-14; previous permission result cannot be reused.</x:v>
       </x:c>
       <x:c r="L57" s="51" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M57" s="51" t="str">
-        <x:v>No Editor login is available.</x:v>
+        <x:v>Editor Capacity Planning navigation is hidden and direct route access is denied.</x:v>
       </x:c>
       <x:c r="N57" s="51" t="str">
         <x:v>https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
       </x:c>
       <x:c r="O57" s="51" t="str">
-        <x:v>No Editor login is available.</x:v>
+        <x:v>Closed by BA confirmation; no DEV fix required.</x:v>
       </x:c>
       <x:c r="P57" s="51" t="str">
-        <x:v>Codex DevInt retest</x:v>
+        <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q57" s="51" t="str">
-        <x:v>Pending BA review</x:v>
+        <x:v>BA confirmed 2026-08-17</x:v>
       </x:c>
       <x:c r="R57" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>46251</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -9284,25 +9348,25 @@
         <x:v>Pass 2026-07-27: FE-318 is owned by Data &amp; Reporting in Portfolio Items and is split across both Teams in CP-001. Its row under Core Platform read From Data &amp; Reporting while its row under Data &amp; Reporting read —, so the column attributes the split to the origin Team and stays silent on the origin's own row. Hover text on each state explains the attribution. Dependencies showed — on every row with a tooltip stating it is not modelled in this slice. Both new columns are read-only. With nine columns the table now scrolls horizontally: measured scrollWidth 1180 against clientWidth 1103, and scrolling to the end revealed the Estimated column intact</x:v>
       </x:c>
       <x:c r="L63" s="51" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M63" s="51" t="str">
-        <x:v>FE-2 own-Team Allocation and Dependencies show 0 instead of —. From Pegasus remains downstream-blocked by P5-CP-006.</x:v>
+        <x:v>Split allocation shows own-Team label "to Retest Capacity", cross-Team label "from Pegasus", and Dependencies may be 0.</x:v>
       </x:c>
       <x:c r="N63" s="51" t="str">
-        <x:v>../Codex_audit_06_tracker.md; https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
+        <x:v>https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
       </x:c>
       <x:c r="O63" s="51" t="str">
-        <x:v>Render — for own-Team Allocation and Dependencies; retest cross-Team origin after P5-CP-006.</x:v>
+        <x:v>Closed by BA confirmation; no DEV fix required.</x:v>
       </x:c>
       <x:c r="P63" s="51" t="str">
         <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q63" s="51" t="str">
-        <x:v>BA confirmed Fail 2026-08-14</x:v>
+        <x:v>BA confirmed 2026-08-17</x:v>
       </x:c>
       <x:c r="R63" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>46251</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -9343,25 +9407,25 @@
         <x:v>Superseded by approved Project access baseline 2026-08-14; previous permission result cannot be reused.</x:v>
       </x:c>
       <x:c r="L64" s="51" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M64" s="51" t="str">
-        <x:v>Only Workspace Admin session is available; fixed Admin/Editor access mapping cannot be verified.</x:v>
+        <x:v>Fixed role/access mapping is enforced; no custom permission matrix is exposed.</x:v>
       </x:c>
       <x:c r="N64" s="51" t="str">
-        <x:v>https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
+        <x:v>https://rally-dev.qnsc.vn/settings</x:v>
       </x:c>
       <x:c r="O64" s="51" t="str">
-        <x:v>Only Workspace Admin session is available; fixed Admin/Editor access mapping cannot be verified.</x:v>
+        <x:v>Closed by BA confirmation; no DEV fix required.</x:v>
       </x:c>
       <x:c r="P64" s="51" t="str">
-        <x:v>Codex DevInt retest</x:v>
+        <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q64" s="51" t="str">
-        <x:v>Pending BA review</x:v>
+        <x:v>BA confirmed 2026-08-17</x:v>
       </x:c>
       <x:c r="R64" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>46251</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
@@ -9407,25 +9471,25 @@
         <x:v>Pass 2026-07-28. Removing FE-318 from Plan cleared it from Core Platform and Data &amp; Reporting, changed both Team Feature counts to 0, removed the Feature text from the plan and recalculated Demand to 0.</x:v>
       </x:c>
       <x:c r="L65" s="51" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M65" s="51" t="str">
-        <x:v>The scenario requires a split Feature across multiple Teams. Its prerequisite cannot be created because Team creation rejects an optional Unassigned Team lead.</x:v>
+        <x:v>Remove from Plan on split FE-2 removed both Team allocations; counters recalculated to 0 and FE-2 disappeared until re-added.</x:v>
       </x:c>
       <x:c r="N65" s="51" t="str">
-        <x:v>DEVINT_RETEST_EXECUTION_PLAN_2026-08-14.md §8; https://rally-dev.qnsc.vn/settings</x:v>
+        <x:v>https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
       </x:c>
       <x:c r="O65" s="51" t="str">
-        <x:v>Blocked by the Team creation defect; no disposable split Feature can be prepared.</x:v>
+        <x:v>Closed after current DevInt retest.</x:v>
       </x:c>
       <x:c r="P65" s="51" t="str">
         <x:v>Codex DevInt retest</x:v>
       </x:c>
       <x:c r="Q65" s="51" t="str">
-        <x:v>Pending BA review</x:v>
-      </x:c>
-      <x:c r="R65" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>Codex retest 2026-08-17</x:v>
+      </x:c>
+      <x:c r="R65" s="56" t="str">
+        <x:v>2026-08-17</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
@@ -9474,22 +9538,22 @@
         <x:v>Fail</x:v>
       </x:c>
       <x:c r="M66" s="51" t="str">
-        <x:v>FE-2 child US-5 has Plan Estimate 3, but Complete/Rollup remain 0 at Idea and Completed after reload. US-5 was restored to Idea.</x:v>
+        <x:v>FE-2 has completed child points totaling 5 but Capacity Planning still shows Complete/Rollup = 0.</x:v>
       </x:c>
       <x:c r="N66" s="51" t="str">
-        <x:v>../Codex_audit_06_tracker.md; https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
+        <x:v>https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
       </x:c>
       <x:c r="O66" s="51" t="str">
-        <x:v>Fix child Plan Estimate aggregation and status rollback recalculation.</x:v>
+        <x:v>DEV: recalculate and persist plan rollup from eligible descendant work items after status/estimate changes; refresh all Team and plan totals from the same rollup source.</x:v>
       </x:c>
       <x:c r="P66" s="51" t="str">
         <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q66" s="51" t="str">
-        <x:v>BA confirmed Fail 2026-08-14</x:v>
+        <x:v>BA confirmed 2026-08-17</x:v>
       </x:c>
       <x:c r="R66" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>46251</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
@@ -9534,25 +9598,25 @@
         <x:v>Pass 2026-07-28. Seeded Data &amp; Reporting row (Rollup 6, Estimated 5) displayed the warning triangle and tooltip text; the expanded FE-318 row under Data &amp; Reporting also displayed Rollup exceeds Estimated. Tooltip used fixed overlay and was not clipped by the grid. Build passed with only the standard Vite chunk-size warning.</x:v>
       </x:c>
       <x:c r="L67" s="51" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="M67" s="51" t="str">
-        <x:v>Missing-estimate and Estimated-over-Capacity warnings pass. Rollup warnings are blocked by P5-CP-029 and cross-Team warnings by P5-CP-006; Capacity was restored to 20.</x:v>
+        <x:v>Estimated greater than Capacity warnings and advisory UI work; rollup-dependent warning cannot be confirmed because P5-CP-029 remains open.</x:v>
       </x:c>
       <x:c r="N67" s="51" t="str">
-        <x:v>../Codex_audit_06_tracker.md; https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
+        <x:v>https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
       </x:c>
       <x:c r="O67" s="51" t="str">
-        <x:v>Retest Rollup and cross-Team warning branches after P5-CP-029 and P5-CP-006 are fixed.</x:v>
+        <x:v>DEV: retest the rollup warning branch after P5-CP-029 is fixed; do not change the accepted capacity warning behavior.</x:v>
       </x:c>
       <x:c r="P67" s="51" t="str">
         <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q67" s="51" t="str">
-        <x:v>BA confirmed Fail 2026-08-14</x:v>
+        <x:v>BA confirmed 2026-08-17</x:v>
       </x:c>
       <x:c r="R67" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>46251</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
@@ -9661,25 +9725,25 @@
         <x:v>Pass 2026-07-28. Browser smoke confirmed FE-315 showed the yellow ⚠ Not assigned combobox with Teams Core Platform, Identity &amp; Access, and Data &amp; Reporting; FE-318 stayed as 2 teams with split allocation subrows and no inline one-Team selector. Build passed with only the standard Vite chunk-size warning.</x:v>
       </x:c>
       <x:c r="L69" s="51" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M69" s="51" t="str">
-        <x:v>BA confirmed live 2026-08-14: Planned Team Assignment is inconsistent with allocation ledger/team rail.</x:v>
+        <x:v>Planned Team Assignment matched the ledger: split FE-2 showed 2 teams with rail 8/20 and 2/--; one-Team FE-2 showed Pegasus; removed-Team FE-4 returned to Not assigned.</x:v>
       </x:c>
       <x:c r="N69" s="51" t="str">
         <x:v>https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
       </x:c>
       <x:c r="O69" s="51" t="str">
-        <x:v>FE-2 Planned Team displays `Not assigned` while the same row shows Team Pegasus, estimate `Allocated 8`, and Team rail 8/30; the selector and allocation ledger disagree.</x:v>
+        <x:v>Closed after current DevInt retest.</x:v>
       </x:c>
       <x:c r="P69" s="51" t="str">
         <x:v>Codex DevInt retest</x:v>
       </x:c>
       <x:c r="Q69" s="51" t="str">
-        <x:v>Pending BA review</x:v>
-      </x:c>
-      <x:c r="R69" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>Codex retest 2026-08-17</x:v>
+      </x:c>
+      <x:c r="R69" s="56" t="str">
+        <x:v>2026-08-17</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
@@ -9728,22 +9792,22 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="M70" s="51" t="str">
-        <x:v>Drag/drop Rank, Allocate to Teams, Remove from Plan, Plan Actions placement and Breakdown are accepted. Warning branches remain pending P5-CP-029 and P5-CP-006 fixes.</x:v>
+        <x:v>Ranks, drag/drop, actions, breakdown and plan menu work; rollup-dependent branches remain unverified due to P5-CP-029.</x:v>
       </x:c>
       <x:c r="N70" s="51" t="str">
-        <x:v>../Codex_audit_06_tracker.md; https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
+        <x:v>https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
       </x:c>
       <x:c r="O70" s="51" t="str">
-        <x:v>Retest only the remaining warning branches after upstream fixes.</x:v>
+        <x:v>DEV: retain accepted drag/drop and actions; retest rollup-dependent branches after P5-CP-029 is fixed.</x:v>
       </x:c>
       <x:c r="P70" s="51" t="str">
         <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q70" s="51" t="str">
-        <x:v>BA confirmed Partial 2026-08-14</x:v>
+        <x:v>BA confirmed 2026-08-17</x:v>
       </x:c>
       <x:c r="R70" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>46251</x:v>
       </x:c>
     </x:row>
     <x:row r="71">
@@ -9853,25 +9917,25 @@
         <x:v>DEV/QA acceptance coverage - production API behavior Not Run</x:v>
       </x:c>
       <x:c r="L72" s="51" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="M72" s="51" t="str">
-        <x:v>Full matching and mismatching Release-date publish requires a Feature assigned to a valid Team. Team setup cannot be completed because optional Team lead is rejected.</x:v>
+        <x:v>Publish exact/mismatch core behavior works; advisory wording is incorrect and FE-2 appears duplicated after split allocation.</x:v>
       </x:c>
       <x:c r="N72" s="51" t="str">
-        <x:v>DEVINT_RETEST_EXECUTION_PLAN_2026-08-14.md §8; https://rally-dev.qnsc.vn/settings</x:v>
+        <x:v>https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
       </x:c>
       <x:c r="O72" s="51" t="str">
-        <x:v>Blocked by the Team creation defect; publish date-consistency branches remain untestable.</x:v>
+        <x:v>DEV: use the accepted publish advisory wording and de-duplicate a split Feature in plan review while preserving Team allocations.</x:v>
       </x:c>
       <x:c r="P72" s="51" t="str">
-        <x:v>Codex DevInt retest</x:v>
+        <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q72" s="51" t="str">
-        <x:v>Pending BA review</x:v>
+        <x:v>BA confirmed 2026-08-17</x:v>
       </x:c>
       <x:c r="R72" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>46251</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
@@ -9916,25 +9980,25 @@
         <x:v>Found and fixed 2026-07-27, introduced by the P5-CP-020 change. Widening the picker to all Project Features let a non-Release-matching Feature (FE-308, Q2 2025) be added, but every display lookup still resolved the Feature through eligibleFeatures, which excludes it - so getPlanFeature returned undefined and the row was silently dropped while the allocation still counted in the Team's Features total. Observed as Core Platform reporting Features 3 with only 2 rows rendered. Fixed by resolving all five display lookups against the full Feature list instead of the eligibility-filtered one, with a comment on getPlanFeature recording why an eligibility-filtered list must never be passed there; eligibleFeatures still governs what the plan-level picker offers. Re-verified: FE-308 now renders as a real row (rank 4, value 0) and the Team's Features count matches the rows shown</x:v>
       </x:c>
       <x:c r="L73" s="51" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M73" s="51" t="str">
-        <x:v>A mismatched-Release allocation cannot be added to a Team until valid Team setup works. The required allocation row cannot be produced safely.</x:v>
+        <x:v>FE-4 with no Release was added and allocated to Retest Capacity; its Team expanded row remained visible.</x:v>
       </x:c>
       <x:c r="N73" s="51" t="str">
-        <x:v>DEVINT_RETEST_EXECUTION_PLAN_2026-08-14.md §8; https://rally-dev.qnsc.vn/settings</x:v>
+        <x:v>https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
       </x:c>
       <x:c r="O73" s="51" t="str">
-        <x:v>Blocked by the Team creation defect; retest row visibility after Team setup is fixed.</x:v>
+        <x:v>Closed after current DevInt retest.</x:v>
       </x:c>
       <x:c r="P73" s="51" t="str">
         <x:v>Codex DevInt retest</x:v>
       </x:c>
       <x:c r="Q73" s="51" t="str">
-        <x:v>Pending BA review</x:v>
-      </x:c>
-      <x:c r="R73" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>Codex retest 2026-08-17</x:v>
+      </x:c>
+      <x:c r="R73" s="56" t="str">
+        <x:v>2026-08-17</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
@@ -10728,25 +10792,25 @@
         <x:v>Superseded by approved Project access baseline 2026-08-14; previous permission result cannot be reused.</x:v>
       </x:c>
       <x:c r="L8" s="51" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M8" s="51" t="str">
-        <x:v>Workspace Admin can open Release Tracking and all three Reports. No Admin, Editor or unassigned login is available for authorization boundaries.</x:v>
+        <x:v>Workspace Admin and Project Admin can access Reports/Release Tracking; Editor and unassigned users are denied.</x:v>
       </x:c>
       <x:c r="N8" s="51" t="str">
         <x:v>https://rally-dev.qnsc.vn/reports</x:v>
       </x:c>
       <x:c r="O8" s="51" t="str">
-        <x:v>Workspace Admin can open Release Tracking and all three Reports. No Admin, Editor or unassigned login is available for authorization boundaries.</x:v>
+        <x:v>Closed by BA confirmation; no DEV fix required.</x:v>
       </x:c>
       <x:c r="P8" s="51" t="str">
-        <x:v>Codex DevInt retest</x:v>
+        <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q8" s="51" t="str">
-        <x:v>Pending BA review</x:v>
+        <x:v>BA confirmed 2026-08-17</x:v>
       </x:c>
       <x:c r="R8" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>46251</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -11844,25 +11908,25 @@
         <x:v>New production acceptance scenario</x:v>
       </x:c>
       <x:c r="L26" s="51" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M26" s="51" t="str">
-        <x:v>Localhost fixture retest: Sprint 26.1 has 20 finalized snapshot rows across All Teams and Team Alpha, covering 10 distinct dates. The deliberately missing 2026-06-24 remains a null gap instead of being fabricated.</x:v>
+        <x:v>History Sprint renders 2026-08-17 snapshot (Task To Do 4, Ideal 4, Accepted 0) and missing dates as explicit no data gaps.</x:v>
       </x:c>
       <x:c r="N26" s="51" t="str">
-        <x:v>D:\QNSC\Workspace\rally\.codex-runlogs\local-phase6-blocked-harness.ts</x:v>
+        <x:v>https://rally-dev.qnsc.vn/reports</x:v>
       </x:c>
       <x:c r="O26" s="51" t="str">
-        <x:v>Local DB/domain rule passed. Keep Partial until the same scenario is retested through the deployed API/UI on DevInt and survives reload.</x:v>
+        <x:v>Closed after current DevInt retest.</x:v>
       </x:c>
       <x:c r="P26" s="51" t="str">
         <x:v>Codex localhost fixture retest</x:v>
       </x:c>
       <x:c r="Q26" s="51" t="str">
-        <x:v>Local evidence added; DevInt UI retest pending</x:v>
-      </x:c>
-      <x:c r="R26" s="56" t="n">
-        <x:v>46249</x:v>
+        <x:v>Codex retest 2026-08-17</x:v>
+      </x:c>
+      <x:c r="R26" s="56" t="str">
+        <x:v>2026-08-17</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -11911,22 +11975,22 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M27" s="51" t="str">
-        <x:v>No daily snapshots/controlled acceptedDate data exist; mutation is paused after the Work Item Team-clearing defect.</x:v>
+        <x:v>No finalized post-Accept daily snapshot is available; US-17 changed live while the old frozen snapshot remained 0, then was restored to Idea.</x:v>
       </x:c>
       <x:c r="N27" s="51" t="str">
-        <x:v>https://rally-dev.qnsc.vn/reports</x:v>
+        <x:v>https://rally-dev.qnsc.vn/iteration-status</x:v>
       </x:c>
       <x:c r="O27" s="51" t="str">
-        <x:v>No daily snapshots/controlled acceptedDate data exist; mutation is paused after the Work Item Team-clearing defect.</x:v>
+        <x:v>BLOCKED: create/finalize a new daily snapshot after acceptance, then verify frozen snapshot immutability against later edits.</x:v>
       </x:c>
       <x:c r="P27" s="51" t="str">
-        <x:v>Codex DevInt retest</x:v>
+        <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q27" s="51" t="str">
-        <x:v>Pending BA review</x:v>
+        <x:v>BA confirmed 2026-08-17</x:v>
       </x:c>
       <x:c r="R27" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>46251</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -11972,25 +12036,25 @@
         <x:v>New production acceptance scenario</x:v>
       </x:c>
       <x:c r="L28" s="51" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M28" s="51" t="str">
-        <x:v>Localhost fixture retest: changing current Task TA-2 To Do from 3h to 1h did not change any finalized historical snapshot row; the Task value was restored after comparison.</x:v>
+        <x:v>No finalized snapshot D with accepted points exists to compare against reopen activity on D+1.</x:v>
       </x:c>
       <x:c r="N28" s="51" t="str">
-        <x:v>D:\QNSC\Workspace\rally\.codex-runlogs\local-phase6-blocked-harness.ts</x:v>
+        <x:v>https://rally-dev.qnsc.vn/iteration-status</x:v>
       </x:c>
       <x:c r="O28" s="51" t="str">
-        <x:v>Local DB/domain rule passed. Keep Partial until the same scenario is retested through the deployed API/UI on DevInt and survives reload.</x:v>
+        <x:v>BLOCKED: prepare a finalized snapshot on day D and reopen/change the item on D+1 before retest.</x:v>
       </x:c>
       <x:c r="P28" s="51" t="str">
-        <x:v>Codex localhost fixture retest</x:v>
+        <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q28" s="51" t="str">
-        <x:v>Local evidence added; DevInt UI retest pending</x:v>
+        <x:v>BA confirmed 2026-08-17</x:v>
       </x:c>
       <x:c r="R28" s="56" t="n">
-        <x:v>46249</x:v>
+        <x:v>46251</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -12036,25 +12100,25 @@
         <x:v>New production acceptance scenario</x:v>
       </x:c>
       <x:c r="L29" s="51" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M29" s="51" t="str">
-        <x:v>Localhost fixture retest: changing TA-2 Estimate from 3h to 9h left the captured Iteration baseline unchanged at 40h; the Task estimate was restored after comparison.</x:v>
+        <x:v>Changed TA-1 To Do 0→2 after Iteration start; History Sprint retained Task To Do snapshot 4 and Ideal baseline 4. TA-1 was restored to 0.</x:v>
       </x:c>
       <x:c r="N29" s="51" t="str">
-        <x:v>D:\QNSC\Workspace\rally\.codex-runlogs\local-phase6-blocked-harness.ts</x:v>
+        <x:v>https://rally-dev.qnsc.vn/reports</x:v>
       </x:c>
       <x:c r="O29" s="51" t="str">
-        <x:v>Local DB/domain rule passed. Keep Partial until the same scenario is retested through the deployed API/UI on DevInt and survives reload.</x:v>
+        <x:v>Closed after current DevInt retest.</x:v>
       </x:c>
       <x:c r="P29" s="51" t="str">
         <x:v>Codex localhost fixture retest</x:v>
       </x:c>
       <x:c r="Q29" s="51" t="str">
-        <x:v>Local evidence added; DevInt UI retest pending</x:v>
-      </x:c>
-      <x:c r="R29" s="56" t="n">
-        <x:v>46249</x:v>
+        <x:v>Codex retest 2026-08-17</x:v>
+      </x:c>
+      <x:c r="R29" s="56" t="str">
+        <x:v>2026-08-17</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -12099,25 +12163,25 @@
         <x:v>New production acceptance scenario</x:v>
       </x:c>
       <x:c r="L30" s="51" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M30" s="51" t="str">
-        <x:v>Localhost fixture retest: latest Remaining To Do 0h versus Ideal 0h returns On track; a controlled 1h versus Ideal 0h returns Behind plan.</x:v>
+        <x:v>Latest available row reports Remaining Task To Do 4 versus Ideal 4 and status On track.</x:v>
       </x:c>
       <x:c r="N30" s="51" t="str">
-        <x:v>D:\QNSC\Workspace\rally\.codex-runlogs\local-phase6-blocked-harness.ts</x:v>
+        <x:v>https://rally-dev.qnsc.vn/reports</x:v>
       </x:c>
       <x:c r="O30" s="51" t="str">
-        <x:v>Local DB/domain rule passed. Keep Partial until the same scenario is retested through the deployed API/UI on DevInt and survives reload.</x:v>
+        <x:v>Closed after current DevInt retest.</x:v>
       </x:c>
       <x:c r="P30" s="51" t="str">
         <x:v>Codex localhost fixture retest</x:v>
       </x:c>
       <x:c r="Q30" s="51" t="str">
-        <x:v>Local evidence added; DevInt UI retest pending</x:v>
-      </x:c>
-      <x:c r="R30" s="56" t="n">
-        <x:v>46249</x:v>
+        <x:v>Codex retest 2026-08-17</x:v>
+      </x:c>
+      <x:c r="R30" s="56" t="str">
+        <x:v>2026-08-17</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -12162,25 +12226,25 @@
         <x:v>New production acceptance scenario</x:v>
       </x:c>
       <x:c r="L31" s="51" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M31" s="51" t="str">
-        <x:v>Localhost fixture retest: All Teams and Team Alpha each contain 10 aligned historical dates with identical measured Remaining To Do and Accepted Points; no duplicate aggregate rows were introduced.</x:v>
+        <x:v>Pegasus and All Teams show the same five dates and identical 2026-08-17 values 4/4/0 without duplicate aggregation.</x:v>
       </x:c>
       <x:c r="N31" s="51" t="str">
-        <x:v>D:\QNSC\Workspace\rally\.codex-runlogs\local-phase6-blocked-harness.ts</x:v>
+        <x:v>https://rally-dev.qnsc.vn/reports</x:v>
       </x:c>
       <x:c r="O31" s="51" t="str">
-        <x:v>Local DB/domain rule passed. Keep Partial until the same scenario is retested through the deployed API/UI on DevInt and survives reload.</x:v>
+        <x:v>Closed after current DevInt retest.</x:v>
       </x:c>
       <x:c r="P31" s="51" t="str">
         <x:v>Codex localhost fixture retest</x:v>
       </x:c>
       <x:c r="Q31" s="51" t="str">
-        <x:v>Local evidence added; DevInt UI retest pending</x:v>
-      </x:c>
-      <x:c r="R31" s="56" t="n">
-        <x:v>46249</x:v>
+        <x:v>Codex retest 2026-08-17</x:v>
+      </x:c>
+      <x:c r="R31" s="56" t="str">
+        <x:v>2026-08-17</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -12350,25 +12414,25 @@
         <x:v>New production acceptance scenario</x:v>
       </x:c>
       <x:c r="L34" s="51" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M34" s="51" t="str">
-        <x:v>Created IT-5 P56-AUDIT After Sprint with US-15 and US-16. Velocity shows 0 During / 3 After / 2 Not Accepted. IT-4 P56-AUDIT During Sprint and US-14 are accepted on 2026-08-15, but the Iteration is not eligible in the completed window until its end date has passed.</x:v>
+        <x:v>All Teams Velocity shows all three segments with controlled rows: During Sprint 5/0/0, After Sprint 0/3/2, Carryover 0/0/8.</x:v>
       </x:c>
       <x:c r="N34" s="51" t="str">
-        <x:v>https://rally-dev.qnsc.vn/reports; https://rally-dev.qnsc.vn/item/US-14; https://rally-dev.qnsc.vn/item/US-15; https://rally-dev.qnsc.vn/item/US-16</x:v>
+        <x:v>https://rally-dev.qnsc.vn/reports</x:v>
       </x:c>
       <x:c r="O34" s="51" t="str">
-        <x:v>Retest the During segment on 2026-08-16, or use a controlled historical acceptedDate fixture. After and Not Accepted branches pass.</x:v>
+        <x:v>Closed after current DevInt retest.</x:v>
       </x:c>
       <x:c r="P34" s="51" t="str">
         <x:v>Codex DevInt retest</x:v>
       </x:c>
       <x:c r="Q34" s="51" t="str">
-        <x:v>Pending BA review</x:v>
-      </x:c>
-      <x:c r="R34" s="56" t="n">
-        <x:v>46249</x:v>
+        <x:v>Codex retest 2026-08-17</x:v>
+      </x:c>
+      <x:c r="R34" s="56" t="str">
+        <x:v>2026-08-17</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -12478,25 +12542,25 @@
         <x:v>New production acceptance scenario</x:v>
       </x:c>
       <x:c r="L36" s="51" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="M36" s="51" t="str">
-        <x:v>Moving shared Work Items is unsafe after the Team-clearing Save defect; no disposable completed iteration exists.</x:v>
+        <x:v>Moving US-2 out of Carryover changes Not Accepted from 8 to 3; completed Carryover cannot be selected to move it back. US-2 remains in Backlog.</x:v>
       </x:c>
       <x:c r="N36" s="51" t="str">
-        <x:v>https://rally-dev.qnsc.vn/reports</x:v>
+        <x:v>https://rally-dev.qnsc.vn/backlog</x:v>
       </x:c>
       <x:c r="O36" s="51" t="str">
-        <x:v>Moving shared Work Items is unsafe after the Team-clearing Save defect; no disposable completed iteration exists.</x:v>
+        <x:v>DEV: allow users to select completed Iterations in Work Item Iteration dropdown; manual assignment must not auto-change Work Item state.</x:v>
       </x:c>
       <x:c r="P36" s="51" t="str">
-        <x:v>Codex DevInt retest</x:v>
+        <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q36" s="51" t="str">
-        <x:v>Pending BA review</x:v>
+        <x:v>BA confirmed 2026-08-17</x:v>
       </x:c>
       <x:c r="R36" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>46251</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -12732,25 +12796,25 @@
         <x:v>New production acceptance scenario</x:v>
       </x:c>
       <x:c r="L40" s="51" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Blocked</x:v>
       </x:c>
       <x:c r="M40" s="51" t="str">
-        <x:v>Localhost fixture retest: US-3 is Accepted with 8 points and acceptedDate = null. Velocity classifies all 8 points as unclassified with unclassifiedItems = 1 and does not guess During or After.</x:v>
+        <x:v>Direct Idea to Release stamps acceptedDate and classifies After; shared DevInt cannot safely create an invalid Accepted/Release record with null acceptedDate. US-1 was restored to Idea.</x:v>
       </x:c>
       <x:c r="N40" s="51" t="str">
-        <x:v>D:\QNSC\Workspace\rally\.codex-runlogs\local-phase6-blocked-harness.ts</x:v>
+        <x:v>https://rally-dev.qnsc.vn/item/US-1</x:v>
       </x:c>
       <x:c r="O40" s="51" t="str">
-        <x:v>Local DB/domain rule passed. Keep Partial until the same scenario is retested through the deployed API/UI on DevInt and survives reload.</x:v>
+        <x:v>BLOCKED/DEV TEST: use a localhost fixture or controlled migration test with Accepted/Release plus null acceptedDate and verify fallback classification.</x:v>
       </x:c>
       <x:c r="P40" s="51" t="str">
-        <x:v>Codex localhost fixture retest</x:v>
+        <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q40" s="51" t="str">
-        <x:v>Local evidence added; DevInt UI retest pending</x:v>
+        <x:v>BA confirmed 2026-08-17</x:v>
       </x:c>
       <x:c r="R40" s="56" t="n">
-        <x:v>46249</x:v>
+        <x:v>46251</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -12795,25 +12859,25 @@
         <x:v>New production acceptance scenario</x:v>
       </x:c>
       <x:c r="L41" s="51" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M41" s="51" t="str">
-        <x:v>Pegasus and All Teams return the same single-Team 0/0/8 result; multi-Team alignment and duplicate-ID prevention cannot be proved.</x:v>
+        <x:v>Pegasus and All Teams overlap on Carryover Sprint with identical 0 During, 0 After, 8 Not Accepted; All Teams adds other Iterations once each.</x:v>
       </x:c>
       <x:c r="N41" s="51" t="str">
         <x:v>https://rally-dev.qnsc.vn/reports</x:v>
       </x:c>
       <x:c r="O41" s="51" t="str">
-        <x:v>Pegasus and All Teams return the same single-Team 0/0/8 result; multi-Team alignment and duplicate-ID prevention cannot be proved.</x:v>
+        <x:v>Closed after current DevInt retest.</x:v>
       </x:c>
       <x:c r="P41" s="51" t="str">
         <x:v>Codex DevInt retest</x:v>
       </x:c>
       <x:c r="Q41" s="51" t="str">
-        <x:v>Pending BA review</x:v>
-      </x:c>
-      <x:c r="R41" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>Codex retest 2026-08-17</x:v>
+      </x:c>
+      <x:c r="R41" s="56" t="str">
+        <x:v>2026-08-17</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -13286,25 +13350,25 @@
         <x:v>New production acceptance scenario</x:v>
       </x:c>
       <x:c r="L49" s="51" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M49" s="51" t="str">
-        <x:v>BA confirmed live 2026-08-14: null-owner Task hours are attributed to a named member.</x:v>
+        <x:v>TA-3 under Unassigned shows Capacity 0, Estimate 4, To Do 4 and Actual 0; no named member receives the hours.</x:v>
       </x:c>
       <x:c r="N49" s="51" t="str">
-        <x:v>DEVINT_RETEST_EXECUTION_PLAN_2026-08-14.md §8; https://rally-dev.qnsc.vn/reports</x:v>
+        <x:v>https://rally-dev.qnsc.vn/team-status</x:v>
       </x:c>
       <x:c r="O49" s="51" t="str">
-        <x:v>Fail: an unassigned Task must not be attributed to a named member; use the Unassigned group defined by the report rule.</x:v>
+        <x:v>Closed by BA confirmation; no DEV fix required.</x:v>
       </x:c>
       <x:c r="P49" s="51" t="str">
-        <x:v>Codex DevInt retest</x:v>
+        <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q49" s="51" t="str">
-        <x:v>Pending BA review</x:v>
+        <x:v>BA confirmed 2026-08-17</x:v>
       </x:c>
       <x:c r="R49" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>46251</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -13349,25 +13413,25 @@
         <x:v>New production acceptance scenario</x:v>
       </x:c>
       <x:c r="L50" s="51" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M50" s="51" t="str">
-        <x:v>Business rule updated 2026-08-14; the prior formula-based result is obsolete and requires retest.</x:v>
+        <x:v>Team Capacity reflected independently edited Task values (Estimate 4, To Do 2, Actual 0) without recalculating Estimate; Task was restored to To Do 0.</x:v>
       </x:c>
       <x:c r="N50" s="51" t="str">
-        <x:v>DEVINT_RETEST_EXECUTION_PLAN_2026-08-14.md §8; https://rally-dev.qnsc.vn/item/US-9; https://rally-dev.qnsc.vn/reports</x:v>
+        <x:v>https://rally-dev.qnsc.vn/reports</x:v>
       </x:c>
       <x:c r="O50" s="51" t="str">
-        <x:v>Fail: Estimate must be read-only and recomputed to 2h when To Do = 0h and Actual = 2h.</x:v>
+        <x:v>Closed after current DevInt retest.</x:v>
       </x:c>
       <x:c r="P50" s="51" t="str">
         <x:v>Codex DevInt retest</x:v>
       </x:c>
       <x:c r="Q50" s="51" t="str">
-        <x:v>Pending BA review</x:v>
-      </x:c>
-      <x:c r="R50" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>Codex retest 2026-08-17</x:v>
+      </x:c>
+      <x:c r="R50" s="56" t="str">
+        <x:v>2026-08-17</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -13728,25 +13792,25 @@
         <x:v>New production acceptance scenario</x:v>
       </x:c>
       <x:c r="L56" s="51" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M56" s="51" t="str">
-        <x:v>Under AUDIT26, Work Item US-1 exposed TEST Release RE-1 and TEST Team/Task roll-up values while Project remained AUDIT26. Valid Iterations were unavailable; Release Tracking route isolation itself passed.</x:v>
+        <x:v>Selecting AUDIT26 then opening global US-1 switched context to its owning TEST project; Project, Team, Iteration, Task roll-up and Release remained TEST-consistent with no mixed-project values.</x:v>
       </x:c>
       <x:c r="N56" s="51" t="str">
-        <x:v>../Codex_audit_06_tracker.md; https://rally-dev.qnsc.vn/item/US-1; https://rally-dev.qnsc.vn/release-tracking</x:v>
+        <x:v>https://rally-dev.qnsc.vn/item/US-1</x:v>
       </x:c>
       <x:c r="O56" s="51" t="str">
-        <x:v>Scope Work Item relationship queries and late responses by active Project; prevent cross-Project Release, Iteration, Team, Feature and Task data leakage.</x:v>
+        <x:v>Closed after current DevInt retest.</x:v>
       </x:c>
       <x:c r="P56" s="51" t="str">
         <x:v>BA + Codex</x:v>
       </x:c>
       <x:c r="Q56" s="51" t="str">
-        <x:v>BA confirmed Fail 2026-08-14</x:v>
-      </x:c>
-      <x:c r="R56" s="56" t="n">
-        <x:v>46248</x:v>
+        <x:v>Codex retest 2026-08-17</x:v>
+      </x:c>
+      <x:c r="R56" s="56" t="str">
+        <x:v>2026-08-17</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -13845,7 +13909,7 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="4" t="str">
+      <x:c r="A1" s="121" t="str">
         <x:v>Execution Run Log</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
@@ -13858,7 +13922,7 @@
       <x:c r="I1" s="4"/>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
-      <x:c r="A2" s="8" t="str">
+      <x:c r="A2" s="122" t="str">
         <x:v>Append one row per executed scenario. Keep evidence paths relative to 07_Testing Plan/02_test_phase_5_6.</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
@@ -13870,8 +13934,11 @@
       <x:c r="H2" s="8"/>
       <x:c r="I2" s="8"/>
     </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="92"/>
+    </x:row>
     <x:row r="4">
-      <x:c r="A4" s="12" t="str">
+      <x:c r="A4" s="124" t="str">
         <x:v>Date</x:v>
       </x:c>
       <x:c r="B4" s="12" t="str">
@@ -15731,15 +15798,33 @@
       </x:c>
     </x:row>
     <x:row r="72">
-      <x:c r="A72" s="86"/>
-      <x:c r="B72" s="83"/>
-      <x:c r="C72" s="83"/>
-      <x:c r="D72" s="83"/>
-      <x:c r="E72" s="83"/>
-      <x:c r="F72" s="83"/>
-      <x:c r="G72" s="83"/>
-      <x:c r="H72" s="83"/>
-      <x:c r="I72" s="73"/>
+      <x:c r="A72" s="86" t="n">
+        <x:v>46251</x:v>
+      </x:c>
+      <x:c r="B72" s="83" t="str">
+        <x:v>BA-RETEST-20260817-FINAL</x:v>
+      </x:c>
+      <x:c r="C72" s="83" t="str">
+        <x:v>https://rally-dev.qnsc.vn/</x:v>
+      </x:c>
+      <x:c r="D72" s="83" t="str">
+        <x:v>Phase 0-6 selected retest</x:v>
+      </x:c>
+      <x:c r="E72" s="83" t="str">
+        <x:v>BA + Codex</x:v>
+      </x:c>
+      <x:c r="F72" s="83" t="str">
+        <x:v>19 Pass / 5 Partial / 5 Fail / 3 Blocked; plus new GAP-P2-IS-004 Fail</x:v>
+      </x:c>
+      <x:c r="G72" s="83" t="str">
+        <x:v>07_Testing Plan/03_Retest/DEVINT_RETEST_CONFIRMATION_PLAN_2026-08-17.md</x:v>
+      </x:c>
+      <x:c r="H72" s="83" t="str">
+        <x:v>6 current Fail</x:v>
+      </x:c>
+      <x:c r="I72" s="73" t="str">
+        <x:v>All 32 targeted cases BA-confirmed; one separate Dev Owner persistence defect added. Final active total: Pass 166; Fail 6; Partial 5; Blocked 3; Not Run 0. SRS Phase 0-6 updated.</x:v>
+      </x:c>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="86"/>
@@ -17262,7 +17347,7 @@
         <x:v>Access changes: next sign-in; company disable/removal: next refresh</x:v>
       </x:c>
       <x:c r="H5" s="118" t="str">
-        <x:v>Approved baseline</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="158.39999389648438" hidden="0" customHeight="1">
@@ -17288,7 +17373,7 @@
         <x:v>Next sign-in</x:v>
       </x:c>
       <x:c r="H6" s="119" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="132" hidden="0" customHeight="1">
@@ -17314,7 +17399,7 @@
         <x:v>Next sign-in</x:v>
       </x:c>
       <x:c r="H7" s="119" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Fail</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="52.79999923706055" hidden="0" customHeight="1">
@@ -17340,7 +17425,7 @@
         <x:v>Immediately after removal; effective session checked on next sign-in</x:v>
       </x:c>
       <x:c r="H8" s="119" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Fail</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="66" hidden="0" customHeight="1">
@@ -17425,10 +17510,12 @@
         <x:v>Only Workspace Admin, Admin and Editor are shown; no editable matrix; Viewer/selectable No Access are absent</x:v>
       </x:c>
       <x:c r="F13" s="112" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="G13" s="112" t="str"/>
-      <x:c r="H13" s="112" t="str"/>
+      <x:c r="H13" s="112" t="str">
+        <x:v>Retested and BA-confirmed on 2026-08-17.</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A14" s="116" t="str">
@@ -17447,10 +17534,12 @@
         <x:v>WA detail is read-only and WA is excluded from Project member lists</x:v>
       </x:c>
       <x:c r="F14" s="113" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="G14" s="113" t="str"/>
-      <x:c r="H14" s="113" t="str"/>
+      <x:c r="H14" s="113" t="str">
+        <x:v>Retested and BA-confirmed on 2026-08-17.</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="92.4000015258789" hidden="0" customHeight="1">
       <x:c r="A15" s="116" t="str">
@@ -17469,10 +17558,12 @@
         <x:v>Project B remains hidden/denied until WA assigns Admin or Editor</x:v>
       </x:c>
       <x:c r="F15" s="113" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="G15" s="113" t="str"/>
-      <x:c r="H15" s="113" t="str"/>
+      <x:c r="H15" s="113" t="str">
+        <x:v>Retested and BA-confirmed on 2026-08-17.</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="92.4000015258789" hidden="0" customHeight="1">
       <x:c r="A16" s="116" t="str">
@@ -17491,10 +17582,12 @@
         <x:v>All Teams and delivery administration are available</x:v>
       </x:c>
       <x:c r="F16" s="113" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="G16" s="113" t="str"/>
-      <x:c r="H16" s="113" t="str"/>
+      <x:c r="H16" s="113" t="str">
+        <x:v>Retested and BA-confirmed on 2026-08-17.</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="105.5999984741211" hidden="0" customHeight="1">
       <x:c r="A17" s="116" t="str">
@@ -17513,10 +17606,12 @@
         <x:v>Project Details, Teams and Users &amp; Permissions are read-only</x:v>
       </x:c>
       <x:c r="F17" s="113" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="G17" s="113" t="str"/>
-      <x:c r="H17" s="113" t="str"/>
+      <x:c r="H17" s="113" t="str">
+        <x:v>Retested and BA-confirmed on 2026-08-17.</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="105.5999984741211" hidden="0" customHeight="1">
       <x:c r="A18" s="116" t="str">
@@ -17535,10 +17630,12 @@
         <x:v>CRUD delivery items only in Team 1; no structural admin, Portfolio, Capacity or Reports</x:v>
       </x:c>
       <x:c r="F18" s="113" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Fail</x:v>
       </x:c>
       <x:c r="G18" s="113" t="str"/>
-      <x:c r="H18" s="113" t="str"/>
+      <x:c r="H18" s="113" t="str">
+        <x:v>Editor Team/project scope leak confirmed on 2026-08-17.</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="92.4000015258789" hidden="0" customHeight="1">
       <x:c r="A19" s="116" t="str">
@@ -17557,10 +17654,12 @@
         <x:v>Project B is absent and direct navigation is safely denied without metadata leak</x:v>
       </x:c>
       <x:c r="F19" s="113" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Fail</x:v>
       </x:c>
       <x:c r="G19" s="113" t="str"/>
-      <x:c r="H19" s="113" t="str"/>
+      <x:c r="H19" s="113" t="str">
+        <x:v>Unassigned metadata/stale context leak confirmed on 2026-08-17.</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="79.19999694824219" hidden="0" customHeight="1">
       <x:c r="A20" s="116" t="str">
@@ -17579,10 +17678,12 @@
         <x:v>Assignment row and Team scope are removed; Project becomes hidden/direct access denied</x:v>
       </x:c>
       <x:c r="F20" s="113" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="G20" s="113" t="str"/>
-      <x:c r="H20" s="113" t="str"/>
+      <x:c r="H20" s="113" t="str">
+        <x:v>Retested and BA-confirmed on 2026-08-17.</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="105.5999984741211" hidden="0" customHeight="1">
       <x:c r="A21" s="116" t="str">
@@ -17601,10 +17702,12 @@
         <x:v>Both journeys show the same Admin/Editor assignment and Team state</x:v>
       </x:c>
       <x:c r="F21" s="113" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="G21" s="113" t="str"/>
-      <x:c r="H21" s="113" t="str"/>
+      <x:c r="H21" s="113" t="str">
+        <x:v>Retested and BA-confirmed on 2026-08-17.</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="92.4000015258789" hidden="0" customHeight="1">
       <x:c r="A22" s="116" t="str">
@@ -17623,10 +17726,12 @@
         <x:v>Admin receives All Teams; Editor joins the selected Team</x:v>
       </x:c>
       <x:c r="F22" s="113" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="G22" s="113" t="str"/>
-      <x:c r="H22" s="113" t="str"/>
+      <x:c r="H22" s="113" t="str">
+        <x:v>Retested and BA-confirmed on 2026-08-17.</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A23" s="117" t="str">

</xml_diff>